<commit_message>
chore: refresh project workbook
</commit_message>
<xml_diff>
--- a/sources/Public Invention Projects.xlsx
+++ b/sources/Public Invention Projects.xlsx
@@ -3546,7 +3546,7 @@
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>Stale</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="C39" s="7" t="s">
@@ -4354,7 +4354,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>August 2026</t>
+          <t>September 2026</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -4480,7 +4480,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>August 2026</t>
+          <t>September 2026</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="B4" s="46" t="inlineStr">
         <is>
-          <t>Stale</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="C4" s="7" t="s">

</xml_diff>

<commit_message>
Stop the refresh overwriting the human Status column, and restore it
</commit_message>
<xml_diff>
--- a/sources/Public Invention Projects.xlsx
+++ b/sources/Public Invention Projects.xlsx
@@ -1854,7 +1854,7 @@
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Ready-to-start</t>
         </is>
       </c>
       <c r="C2" s="7" t="s">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C3" s="7" t="s">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -1946,7 +1946,7 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C4" s="7" t="s">
@@ -1972,7 +1972,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -1992,7 +1992,7 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C5" s="7" t="s">
@@ -2018,7 +2018,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C6" s="7" t="s">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -2084,7 +2084,7 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C7" s="7" t="s">
@@ -2110,7 +2110,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C8" s="7" t="s">
@@ -2156,7 +2156,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C9" s="7" t="s">
@@ -2202,7 +2202,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -2222,7 +2222,7 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C10" s="7" t="s">
@@ -2248,7 +2248,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Highly Active</t>
         </is>
       </c>
       <c r="C11" s="7" t="s">
@@ -2320,7 +2320,7 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C12" s="7" t="s">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C13" s="7" t="s">
@@ -2398,7 +2398,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -2418,7 +2418,7 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Ready-to-start</t>
         </is>
       </c>
       <c r="C14" s="7" t="s">
@@ -2444,7 +2444,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Ready-to-start</t>
         </is>
       </c>
       <c r="C15" s="7" t="s">
@@ -2510,7 +2510,7 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Highly Active</t>
         </is>
       </c>
       <c r="C16" s="7" t="s">
@@ -2542,7 +2542,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2562,7 +2562,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C17" s="7" t="s">
@@ -2588,7 +2588,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Highly Active</t>
         </is>
       </c>
       <c r="C18" s="7" t="s">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Highly Active</t>
         </is>
       </c>
       <c r="C19" s="7" t="s">
@@ -2712,7 +2712,7 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Ready-to-start</t>
         </is>
       </c>
       <c r="C20" s="7" t="s">
@@ -2738,7 +2738,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Ready-to-start</t>
         </is>
       </c>
       <c r="C21" s="7" t="s">
@@ -2784,7 +2784,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2804,7 +2804,7 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Ready-to-start</t>
         </is>
       </c>
       <c r="C22" s="7" t="s">
@@ -2830,7 +2830,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2850,7 +2850,7 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Ready-to-start</t>
         </is>
       </c>
       <c r="C23" s="7" t="s">
@@ -2876,7 +2876,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2896,7 +2896,7 @@
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C24" s="7" t="s">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2942,7 +2942,7 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C25" s="7" t="s">
@@ -2968,7 +2968,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Ready-to-start</t>
         </is>
       </c>
       <c r="C26" s="7" t="s">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Ready-to-start</t>
         </is>
       </c>
       <c r="C27" s="7" t="s">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C28" s="7" t="s">
@@ -3124,7 +3124,7 @@
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C29" s="7" t="s">
@@ -3150,7 +3150,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3170,7 +3170,7 @@
       </c>
       <c r="B30" s="15" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Highly Active</t>
         </is>
       </c>
       <c r="C30" s="7" t="s">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Ready-to-start</t>
         </is>
       </c>
       <c r="C31" s="7" t="s">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -3268,7 +3268,7 @@
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C32" s="7" t="s">
@@ -3294,7 +3294,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="B33" s="15" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Progress but Inactive</t>
         </is>
       </c>
       <c r="C33" s="7" t="s">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Ready-to-start</t>
         </is>
       </c>
       <c r="C34" s="7" t="s">
@@ -3386,7 +3386,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -3406,7 +3406,7 @@
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Ready-to-start</t>
         </is>
       </c>
       <c r="C35" s="7" t="s">
@@ -3448,7 +3448,7 @@
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Ready-to-start</t>
         </is>
       </c>
       <c r="C37" s="7" t="s">
@@ -3474,7 +3474,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -3494,7 +3494,7 @@
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Highly Active</t>
         </is>
       </c>
       <c r="C38" s="7" t="s">
@@ -3546,7 +3546,7 @@
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Highly Active</t>
         </is>
       </c>
       <c r="C39" s="7" t="s">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Stale</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="B40" s="15" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Progress but Inactive</t>
         </is>
       </c>
       <c r="C40" s="7" t="s">
@@ -3640,7 +3640,7 @@
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C41" s="7" t="s">
@@ -3680,7 +3680,7 @@
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C42" s="7" t="s">
@@ -3720,7 +3720,7 @@
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C43" s="7" t="s">
@@ -3760,7 +3760,7 @@
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C44" s="7" t="s">
@@ -3781,7 +3781,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -3801,7 +3801,7 @@
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Highly Active</t>
         </is>
       </c>
       <c r="C45" s="7" t="s">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -3853,7 +3853,7 @@
       </c>
       <c r="B46" s="15" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Progress but Inactive</t>
         </is>
       </c>
       <c r="C46" s="7" t="s">
@@ -3905,7 +3905,7 @@
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C47" s="7" t="s">
@@ -3951,7 +3951,7 @@
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Ready-to-start</t>
         </is>
       </c>
       <c r="C48" s="7" t="s">
@@ -3977,7 +3977,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -3997,7 +3997,7 @@
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C49" s="7" t="s">
@@ -4023,7 +4023,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C50" s="7" t="s">
@@ -4069,7 +4069,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
@@ -4089,7 +4089,7 @@
       </c>
       <c r="B51" s="15" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Progress but Inactive</t>
         </is>
       </c>
       <c r="C51" s="7" t="s">
@@ -4135,7 +4135,7 @@
       </c>
       <c r="B52" s="15" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Progress but Inactive</t>
         </is>
       </c>
       <c r="C52" s="7" t="s">
@@ -4179,7 +4179,7 @@
       </c>
       <c r="B53" s="15" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C53" s="7" t="s">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B54" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C54" s="7" t="s">
@@ -4249,7 +4249,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
@@ -4269,7 +4269,7 @@
       </c>
       <c r="B55" s="15" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Progress but Inactive</t>
         </is>
       </c>
       <c r="C55" s="7" t="s">
@@ -4317,7 +4317,7 @@
       </c>
       <c r="B56" s="15" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Highly Active</t>
         </is>
       </c>
       <c r="C56" s="7" t="s">
@@ -4369,7 +4369,7 @@
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C57" s="7" t="s">
@@ -4409,7 +4409,7 @@
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C58" s="7" t="s">
@@ -4449,7 +4449,7 @@
       </c>
       <c r="B59" s="15" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Progress but Inactive</t>
         </is>
       </c>
       <c r="C59" s="7" t="s">
@@ -4495,7 +4495,7 @@
       </c>
       <c r="B60" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C60" s="7" t="s">
@@ -4521,7 +4521,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
@@ -4541,7 +4541,7 @@
       </c>
       <c r="B61" s="15" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Progress but Inactive</t>
         </is>
       </c>
       <c r="C61" s="7" t="s">
@@ -4587,7 +4587,7 @@
       </c>
       <c r="B62" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C62" s="7" t="s">
@@ -4613,7 +4613,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
@@ -4633,7 +4633,7 @@
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C63" s="7" t="s">
@@ -4659,7 +4659,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
@@ -4679,7 +4679,7 @@
       </c>
       <c r="B64" s="15" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Progress but Inactive</t>
         </is>
       </c>
       <c r="C64" s="7" t="s">
@@ -4725,7 +4725,7 @@
       </c>
       <c r="B65" s="15" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Highly Active</t>
         </is>
       </c>
       <c r="C65" s="7" t="s">
@@ -4777,7 +4777,7 @@
       </c>
       <c r="B66" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C66" s="7" t="s">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B67" s="15" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Highly Active</t>
         </is>
       </c>
       <c r="C67" s="19" t="s">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="B68" s="8" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C68" s="19" t="s">
@@ -4901,7 +4901,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
@@ -4921,7 +4921,7 @@
       </c>
       <c r="B69" s="15" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Highly Active</t>
         </is>
       </c>
       <c r="C69" s="19" t="s">
@@ -4981,7 +4981,7 @@
       </c>
       <c r="B70" s="8" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Preliminary</t>
         </is>
       </c>
       <c r="C70" s="25" t="s">
@@ -5035,7 +5035,7 @@
       </c>
       <c r="B71" s="15" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Highly Active</t>
         </is>
       </c>
       <c r="C71" s="30" t="s">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B72" s="15" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Highly Active</t>
         </is>
       </c>
       <c r="C72" s="19" t="s">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="B4" s="46" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Highly Active</t>
         </is>
       </c>
       <c r="C4" s="7" t="s">
@@ -7594,7 +7594,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Stale</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -7617,7 +7617,7 @@
       </c>
       <c r="B5" s="46" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Highly Active</t>
         </is>
       </c>
       <c r="C5" s="7" t="s">
@@ -7666,7 +7666,7 @@
       </c>
       <c r="B6" s="46" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Highly Active</t>
         </is>
       </c>
       <c r="C6" s="7" t="s">
@@ -7711,7 +7711,7 @@
       </c>
       <c r="B7" s="46" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Highly Active</t>
         </is>
       </c>
       <c r="C7" s="7" t="s">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="B8" s="46" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Highly Active</t>
         </is>
       </c>
       <c r="C8" s="7" t="s">
@@ -7786,7 +7786,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Dormant</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">

</xml_diff>